<commit_message>
feat: optimize AI auto-scan parallel batching, leader lines with draggable balloons, bubble scaling, and UI improvements
</commit_message>
<xml_diff>
--- a/107-M1457_KichThuoc_XuatBaoCao.xlsx
+++ b/107-M1457_KichThuoc_XuatBaoCao.xlsx
@@ -474,10 +474,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-5
-57.5
-1
-±0.005</t>
+          <t>57.51 ±0.005</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -496,7 +493,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>57.51 ±0.005</t>
+          <t>57.51 ±0.005 (Đã duyệt QA)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -516,8 +513,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>-39.4
-±0.01</t>
+          <t>39.4 ±0.01</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -565,17 +561,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>+0.05</t>
+          <t>+0.01</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-0.05</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>57.63 ±0.05</t>
+          <t>(57.63) ±0.01 REF</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -673,20 +669,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>In
-IL
-DP
-0.008
-8
-±0.001
-v
-D
-NITI</t>
+          <t>UIn ID
+DP0.008 ±0.001
+ID NITI</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.008</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -700,7 +690,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0.0088 ±0.001 DP</t>
+          <t>0.008 ±0.001</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -720,18 +710,20 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4°30′23"</t>
+          <t>4°30'23"</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="n">
-        <v>4</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>4°30'23"</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>4°</t>
+          <t>4°30'23"</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">

</xml_diff>